<commit_message>
Added hypothesis testing with the mean population exercises.
</commit_message>
<xml_diff>
--- a/resources/Part_3_Statistics/S20_L125/4.4.Test-for-the-mean.Population-variance-known-exercise.xlsx
+++ b/resources/Part_3_Statistics/S20_L125/4.4.Test-for-the-mean.Population-variance-known-exercise.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18229"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iliya\Desktop\Statistics Course\Filming\Final excel\Section 4 - Hypothesis testing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\D\GitRepos\StatisticsBAandDS\DataScienceBootcamp\resources\Part_3_Statistics\S20_L125\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9084"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9090"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="5" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Population std</t>
   </si>
@@ -90,14 +90,29 @@
   <si>
     <t>You are given the data from the lesson</t>
   </si>
+  <si>
+    <t>Significance (alpha):</t>
+  </si>
+  <si>
+    <t>buscar z(0,05)</t>
+  </si>
+  <si>
+    <t>z value(1-0,05)=z(0,95)</t>
+  </si>
+  <si>
+    <t>1,65 is lower than 4,67</t>
+  </si>
+  <si>
+    <t>Reject the null hypothesis</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -199,7 +214,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -209,10 +224,10 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -223,7 +238,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -536,36 +551,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:J37"/>
-  <sheetFormatPr defaultRowHeight="11.4" x14ac:dyDescent="0.2"/>
+  <dimension ref="B1:L37"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="1"/>
-    <col min="4" max="4" width="12.33203125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.21875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="1"/>
-    <col min="7" max="7" width="4.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="2.5546875" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.21875" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="11.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="1"/>
+    <col min="4" max="4" width="12.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1"/>
+    <col min="7" max="7" width="4.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.42578125" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B2" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B3" s="7"/>
     </row>
-    <row r="4" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B4" s="7" t="s">
         <v>10</v>
       </c>
@@ -573,7 +588,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
         <v>11</v>
       </c>
@@ -581,12 +596,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="12.6" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:12" ht="12.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B8" s="5">
         <v>117313</v>
       </c>
@@ -604,7 +619,7 @@
         <v>113000</v>
       </c>
     </row>
-    <row r="9" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B9" s="5">
         <v>104002</v>
       </c>
@@ -618,7 +633,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B10" s="5">
         <v>113038</v>
       </c>
@@ -629,13 +644,31 @@
         <f>E9/SQRT(E12)</f>
         <v>2738.6127875258308</v>
       </c>
-    </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="I10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B11" s="5">
         <v>101936</v>
       </c>
-    </row>
-    <row r="12" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+      <c r="I11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B12" s="5">
         <v>84560</v>
       </c>
@@ -643,16 +676,20 @@
         <v>7</v>
       </c>
       <c r="E12" s="9">
+        <f>COUNT(B8:B37)</f>
         <v>30</v>
       </c>
       <c r="G12" s="2"/>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B13" s="5">
         <v>113136</v>
       </c>
-    </row>
-    <row r="14" spans="2:10" ht="12" x14ac:dyDescent="0.25">
+      <c r="K13" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B14" s="5">
         <v>80740</v>
       </c>
@@ -663,13 +700,16 @@
         <f>(E8-J8)/E10</f>
         <v>-4.6737652696411374</v>
       </c>
-    </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="K14" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B15" s="5">
         <v>100536</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B16" s="5">
         <v>105052</v>
       </c>
@@ -679,14 +719,14 @@
         <v>87201</v>
       </c>
     </row>
-    <row r="18" spans="2:5" ht="12" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B18" s="5">
         <v>91986</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="10"/>
     </row>
-    <row r="19" spans="2:5" ht="12" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="5">
         <v>94868</v>
       </c>

</xml_diff>